<commit_message>
Add PDF view of self-evaluation form; widen comments column
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Q5ACSQEbZo2UG3FXP6VSM
</commit_message>
<xml_diff>
--- a/self-evaluation/Self_Evaluation_Form_Sidharth_K.xlsx
+++ b/self-evaluation/Self_Evaluation_Form_Sidharth_K.xlsx
@@ -689,6 +689,7 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.38" customWidth="1" style="55" min="1" max="1"/>
+    <col width="45" customWidth="1" style="55" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -972,7 +973,7 @@
       <c r="X7" s="3" t="n"/>
       <c r="Y7" s="3" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="45" customHeight="1" s="55">
       <c r="A8" s="32" t="inlineStr">
         <is>
           <t>Technical &amp; Functional  Knowledge</t>
@@ -1021,7 +1022,7 @@
       <c r="Y8" s="3" t="n"/>
       <c r="Z8" s="3" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="45" customHeight="1" s="55">
       <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Task Management</t>
@@ -1070,7 +1071,7 @@
       <c r="Y9" s="3" t="n"/>
       <c r="Z9" s="3" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="45" customHeight="1" s="55">
       <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Problem Solving</t>
@@ -1119,7 +1120,7 @@
       <c r="Y10" s="3" t="n"/>
       <c r="Z10" s="3" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="45" customHeight="1" s="55">
       <c r="A11" s="37" t="inlineStr">
         <is>
           <t>Communication</t>
@@ -1168,7 +1169,7 @@
       <c r="Y11" s="3" t="n"/>
       <c r="Z11" s="3" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="45" customHeight="1" s="55">
       <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Quality &amp; Process Adherence</t>
@@ -1217,7 +1218,7 @@
       <c r="Y12" s="3" t="n"/>
       <c r="Z12" s="3" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="45" customHeight="1" s="55">
       <c r="A13" s="32" t="inlineStr">
         <is>
           <t>Accountability &amp; Integrity</t>
@@ -1266,7 +1267,7 @@
       <c r="Y13" s="3" t="n"/>
       <c r="Z13" s="3" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="45" customHeight="1" s="55">
       <c r="A14" s="38" t="inlineStr">
         <is>
           <t>As a Team Member</t>
@@ -1315,7 +1316,7 @@
       <c r="Y14" s="3" t="n"/>
       <c r="Z14" s="3" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="45" customHeight="1" s="55">
       <c r="A15" s="38" t="inlineStr">
         <is>
           <t>Independent Work</t>
@@ -1364,7 +1365,7 @@
       <c r="Y15" s="3" t="n"/>
       <c r="Z15" s="3" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="45" customHeight="1" s="55">
       <c r="A16" s="38" t="inlineStr">
         <is>
           <t>Attendance</t>

</xml_diff>